<commit_message>
Week 2 Kahoot (Danish): fresh non-repeating questions, randomized correct answer
Rework week-02-da.xlsx: no questions repeat the Week-1 Kahoot (LEDs/buttons/
on-start/.hex/horse/football), and the correct answer is spread evenly across
positions A/B/C/D instead of always A. Refresh the image cheat-sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188ZkFnwfCFdngpQqnGxYfa
</commit_message>
<xml_diff>
--- a/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
+++ b/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
@@ -456,60 +456,60 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hvor mange lys (LED) er der på micro:bit'ens forside?</t>
+          <t>Hvilken blok gentager koden igen og igen for evigt?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>on start</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>show number</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>pause</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>forever</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>20</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hvad hedder de to knapper på micro:bit'en?</t>
+          <t>Hvilken blok viser et lille billede som et hjerte eller et ansigt?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A og B</t>
+          <t>show icon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1 og 2</t>
+          <t>show string</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>X og Y</t>
+          <t>radio send</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Op og Ned</t>
+          <t>show number</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -522,126 +522,126 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hvilken blok gentager koden HELE tiden, igen og igen?</t>
+          <t>Hvad gør blokken 'pause (ms)'?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>forever</t>
+          <t>Genstarter boardet</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>on start</t>
+          <t>Tænder for musikken</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>Får programmet til at vente lidt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>show number</t>
+          <t>Sletter al koden</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hvilken blok bruger du til at vise et hjerte?</t>
+          <t>Hvilken blok viser bogstaver og ord?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>show icon</t>
+          <t>show arrow</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>pause</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>show number</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>show string</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>pause</t>
-        </is>
-      </c>
       <c r="F5" t="n">
         <v>20</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Hvad gør blokken 'pause (ms)'?</t>
+          <t>Hvad hedder det gratis website, hvor vi bygger koden?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Venter et lille øjeblik</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sletter skærmen</t>
+          <t>Google Docs</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Spiller en sang</t>
+          <t>Minecraft</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Viser dit navn</t>
+          <t>MakeCode</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>20</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hvor koder man til micro:bit'en?</t>
+          <t>Hvad sker der, når du trykker på ▶️-knappen i MakeCode?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>makecode.microbit.org</t>
+          <t>Programmet kører i simulatoren</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Computeren slukker</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Paint</t>
+          <t>Koden slettes</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Der printes</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -654,93 +654,93 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hvordan får du dit program over på det rigtige board?</t>
+          <t>Hvilken blok kører, når du trykker på knap A?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Download .hex og træk til MICROBIT</t>
+          <t>forever</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Print det på papir</t>
+          <t>on button A pressed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Send en SMS</t>
+          <t>on shake</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tag et billede</t>
+          <t>on start</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>20</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hvilken blok viser bogstaver og ord?</t>
+          <t>Hvad gør blokken 'show leds'?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>show string</t>
+          <t>Sender en besked</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>show number</t>
+          <t>Tænder præcis de lys, du vælger</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>show leds</t>
+          <t>Viser et tal</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>Spiller en sang</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>20</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hjertet skal banke HURTIGERE. Hvad gør du?</t>
+          <t>Hvordan laver man et hjerte, der 'banker'?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gør pausen kortere</t>
+          <t>Skift mellem stort og lille hjerte</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gør pausen længere</t>
+          <t>Ryst boardet</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Fjern forever</t>
+          <t>Sluk lyset</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sluk boardet</t>
+          <t>Tryk på A hele tiden</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -753,40 +753,40 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hvilket ikon er det MINDSTE hjerte?</t>
+          <t>Hvilken bevægelse kan micro:bit'en mærke helt af sig selv?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Small heart</t>
+          <t>Din alder</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Rystelse (shake)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Duck</t>
+          <t>Din yndlingsret</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Din stemmes farve</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>20</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>🎮 Hvilket spil handler om at bygge med firkantede klodser?</t>
+          <t>🎮 I hvilket spil bygger man næsten alt med firkantede klodser?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -801,12 +801,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Mario Kart</t>
+          <t>Tetris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tetris</t>
+          <t>Wordle</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -819,133 +819,133 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>🎉 Hvad råber alle efter 'six...'?</t>
+          <t>🎉 Hvilket tal kommer efter 'six...' i den kendte trend?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>seven!</t>
+          <t>ten</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>eight!</t>
+          <t>four</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>nine!</t>
+          <t>seven</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ten!</t>
+          <t>tolv</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>20</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>🕹️ Hvor laver man 'obbys' og sine egne mini-spil?</t>
+          <t>🕹️ Hvor laver folk deres egne spil og 'obbys'?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Roblox</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Snake</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Pac-Man</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kabale</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>20</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>😹 Hvad er en 'meme'?</t>
+          <t>😹 Hvad kalder man et sjovt billede eller klip, der spredes på nettet?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Et sjovt billede/video man deler</t>
+          <t>En pause</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>En slags kage</t>
+          <t>En pixel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>En micro:bit-blok</t>
+          <t>En meme</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>En knap</t>
+          <t>En variabel</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>20</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>📱 'Skibidi' blev kæmpestort på hvilke apps?</t>
+          <t>📱 'Skibidi' blev mega-populært især på hvilke apps?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Paint</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>YouTube og TikTok</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Word</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Paint</t>
+          <t>Lommeregner</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>20</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 2 Kahoot: put the answer options in Danish too
Translate all answer options to Danish (block-name answers use Danish MakeCode
terms, e.g. "gentag for altid", "vis ikon", "vis tekst"); "6 7" answer set now
uses Danish numbers. Cheat-sheet notes to set the editor language to Dansk.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188ZkFnwfCFdngpQqnGxYfa
</commit_message>
<xml_diff>
--- a/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
+++ b/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
@@ -461,22 +461,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>on start</t>
+          <t>ved start</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>show number</t>
+          <t>vis tal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>pause (ms)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>forever</t>
+          <t>gentag for altid</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -494,12 +494,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>show icon</t>
+          <t>vis ikon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>show string</t>
+          <t>vis tekst</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>show number</t>
+          <t>vis tal</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -560,22 +560,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>show arrow</t>
+          <t>vis pil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>pause (ms)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>show number</t>
+          <t>vis tal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>show string</t>
+          <t>vis tekst</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Der printes</t>
+          <t>Der printes på papir</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -659,22 +659,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>forever</t>
+          <t>gentag for altid</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>on button A pressed</t>
+          <t>da knap A trykkes</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>on shake</t>
+          <t>da rystet</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>on start</t>
+          <t>ved start</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -687,7 +687,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hvad gør blokken 'show leds'?</t>
+          <t>Hvad gør blokken 'vis lys' (show leds)?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ten</t>
+          <t>ti</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>four</t>
+          <t>fire</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>seven</t>
+          <t>syv</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Lommeregner</t>
+          <t>Lommeregneren</t>
         </is>
       </c>
       <c r="F16" t="n">

</xml_diff>

<commit_message>
Week 2 Kahoot: use the real Danish MakeCode block names
Verified block labels in the Danish editor and corrected them: "for altid"
(not "gentag for altid"), "vis nummer", "vis streng", "vis LED'er",
"når programmet starter" (on start), "når der trykkes på knappen A", "på ryst".
So the quiz matches exactly what kids see on screen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188ZkFnwfCFdngpQqnGxYfa
</commit_message>
<xml_diff>
--- a/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
+++ b/microbit-program/autumn-2026/quiz/kahoot-import/week-02-da.xlsx
@@ -461,12 +461,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ved start</t>
+          <t>når programmet starter</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vis tal</t>
+          <t>vis nummer</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>gentag for altid</t>
+          <t>for altid</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -499,17 +499,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>vis tekst</t>
+          <t>vis streng</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>radio send</t>
+          <t>radio send nummer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>vis tal</t>
+          <t>vis nummer</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -570,12 +570,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>vis tal</t>
+          <t>vis nummer</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>vis tekst</t>
+          <t>vis streng</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -659,22 +659,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gentag for altid</t>
+          <t>for altid</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>da knap A trykkes</t>
+          <t>når der trykkes på knappen A</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>da rystet</t>
+          <t>på ryst</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ved start</t>
+          <t>når programmet starter</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -687,7 +687,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hvad gør blokken 'vis lys' (show leds)?</t>
+          <t>Hvad gør blokken 'vis LED'er' (show leds)?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">

</xml_diff>